<commit_message>
update export font format
</commit_message>
<xml_diff>
--- a/path2shock_calculation/output/path2shock_finalV.xlsx
+++ b/path2shock_calculation/output/path2shock_finalV.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -38,6 +38,18 @@
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Inter"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Inter"/>
+      <b val="1"/>
+      <color rgb="FF002060"/>
       <sz val="11"/>
     </font>
     <font>
@@ -80,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -105,7 +117,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -472,17 +487,17 @@
           <t>MMM1</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>20.0 %</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -516,17 +531,17 @@
           <t>MMM11</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>198.0% max</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>972.0% max</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>1746.0% max</t>
         </is>
@@ -555,17 +570,17 @@
       <c r="Z4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>(+13.0 ppts)</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>(+13.0 ppts)</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>(+13.0 ppts)</t>
         </is>
@@ -599,17 +614,17 @@
           <t>MMM20</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>1.2 % to 1.1 %</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>0.4 % to 0.4 %</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>0.2 % to 0.2 %</t>
         </is>
@@ -643,17 +658,17 @@
           <t>MMM2</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>4.3 %</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -687,17 +702,17 @@
           <t>MMM12</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>213.3 peak</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>977.300000000001 peak</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>1764.0 peak</t>
         </is>
@@ -726,17 +741,17 @@
       <c r="Z8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>(+10 ppts)</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>(+3 ppts)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>(+13 ppts)</t>
         </is>
@@ -770,17 +785,17 @@
           <t>MMM21</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>378.0 peak</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>1152.0 peak</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>1900.0 trough</t>
         </is>
@@ -809,17 +824,17 @@
       <c r="Z10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>(-500 bps)</t>
         </is>
@@ -853,17 +868,17 @@
           <t>MMM22</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>396.0 peak</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>1170.0 peak</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>1908.0 trough</t>
         </is>
@@ -892,17 +907,17 @@
       <c r="Z12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>(-700 bps)</t>
         </is>
@@ -936,17 +951,17 @@
           <t>MMM23</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>414.0 peak</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>1188.0 peak</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>1907.0 trough</t>
         </is>
@@ -975,17 +990,17 @@
       <c r="Z14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>(-3400 bps)</t>
         </is>
@@ -1019,17 +1034,17 @@
           <t>MMM25</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>450.0 peak</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>1224.0 peak</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>1980.0 trough</t>
         </is>
@@ -1058,17 +1073,17 @@
       <c r="Z16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>(-500 bps)</t>
         </is>
@@ -1102,17 +1117,17 @@
           <t>MMM13</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>234.0 peak</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>1008.0 peak</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>1782.0 peak</t>
         </is>
@@ -1141,17 +1156,17 @@
       <c r="Z18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>(+1300 bps)</t>
         </is>
@@ -1185,17 +1200,17 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>2.4 %</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1229,17 +1244,17 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>1.7 %</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1273,17 +1288,17 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>1.3 %</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1317,17 +1332,17 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>1.1 %</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1361,17 +1376,17 @@
           <t>M7</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>0.9 %</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1405,17 +1420,17 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>0.8 %</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1449,17 +1464,17 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>0.7 %</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
@@ -1493,17 +1508,17 @@
           <t>M24</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>0.2 %</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>0.1 %</t>
         </is>

</xml_diff>